<commit_message>
Ajuste final de los elementos
</commit_message>
<xml_diff>
--- a/ModeloFInal/resultados/RESUMEN EJECUCIÓN.xlsx
+++ b/ModeloFInal/resultados/RESUMEN EJECUCIÓN.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Desktop\Universidad\TFG\ModeloFinal\resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40695395-4FD2-4D7F-B3BD-70D7EB68C556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C691619-9FD0-44CA-8DF3-012E81B1CE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4048496F-68A2-4F9B-80AB-D81190A15522}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4048496F-68A2-4F9B-80AB-D81190A15522}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" r:id="rId1"/>
+    <sheet name=" MAGIC Gamma Telescope" sheetId="1" r:id="rId1"/>
+    <sheet name="IRIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="42">
   <si>
     <t>Polinomio</t>
   </si>
@@ -61,18 +62,6 @@
     <t>Shmaliy</t>
   </si>
   <si>
-    <t>Suma</t>
-  </si>
-  <si>
-    <t>Promedio</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Recuento</t>
-  </si>
-  <si>
     <t>Lineal/Dense</t>
   </si>
   <si>
@@ -167,13 +156,19 @@
   </si>
   <si>
     <t>shmaliy</t>
+  </si>
+  <si>
+    <t>Tiempo_Promedio(s)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,8 +196,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -244,8 +245,38 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+        <bgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+        <bgColor rgb="FFC6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+        <bgColor rgb="FFF8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -264,6 +295,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -274,7 +320,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
@@ -293,6 +339,57 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="40% - Énfasis6" xfId="5" builtinId="51"/>
@@ -402,8 +499,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="3933825"/>
-          <a:ext cx="7772400" cy="3290831"/>
+          <a:off x="0" y="3949867"/>
+          <a:ext cx="7784933" cy="3290831"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1104,6 +1201,805 @@
         <a:xfrm>
           <a:off x="15439950" y="17059200"/>
           <a:ext cx="7772400" cy="3290831"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>550745</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD02276F-75F1-4911-A65B-FDEBB19885A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5314950" y="0"/>
+          <a:ext cx="5113220" cy="3257550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>96583</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA6B666C-5E73-45BB-9367-AD0488FC60D8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="3619500"/>
+          <a:ext cx="8324850" cy="3525583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>13259</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagen 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59E8E564-AA12-4F2A-ACAF-E5E379BD3EB5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="7077075"/>
+          <a:ext cx="8366684" cy="3543300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>83325</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>63907</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{902D8BB1-4DC2-4B22-B125-2AA75E98C223}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="10560825"/>
+          <a:ext cx="8417332" cy="3564750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>166650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>145342</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Imagen 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F3F863C-7CD5-4AB4-AA13-9DE9F0FFF2E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="14073150"/>
+          <a:ext cx="8496300" cy="3598192"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>152399</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>68451</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Imagen 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59A1E38C-4E5C-4019-A425-9D921ADDEFB3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="17611725"/>
+          <a:ext cx="8505824" cy="3602226"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>738868</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>16292</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>136071</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>19125</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Imagen 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE5C2775-A27E-44E1-9109-0DFF93FBA7C1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8331654" y="3635792"/>
+          <a:ext cx="7779203" cy="3241333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>726943</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>137717</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>124146</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>140550</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Imagen 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE78623A-C2FF-438C-A298-9D12FF1E7DBF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8319729" y="6805217"/>
+          <a:ext cx="7779203" cy="3241333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>10168</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>173417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>169371</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>176250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Imagen 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE166B9A-AD00-4AFA-B179-124236C059BD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8364954" y="10079417"/>
+          <a:ext cx="7779203" cy="3241333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>138396</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>122031</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>297599</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>124864</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Imagen 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{098BF144-30AD-4071-AAFA-81DA2EDD60C3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8493182" y="13266531"/>
+          <a:ext cx="7779203" cy="3241333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>121028</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>174060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>280231</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>176893</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Imagen 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{964C2354-38D7-4E01-B95F-88431A97E3CF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8475814" y="16366560"/>
+          <a:ext cx="7779203" cy="3241333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>54428</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>27215</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>206828</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>27214</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Imagen 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E2BD8C8-4DB8-4593-A13A-4E53E914F38D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16029214" y="3646715"/>
+          <a:ext cx="7772400" cy="3238499"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>27536</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>163607</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>179936</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>163606</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Imagen 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6673D44-FD64-466F-B4B3-A4EA13FB6C5E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16002322" y="6831107"/>
+          <a:ext cx="7772400" cy="3238499"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>82286</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>177535</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>234686</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>177534</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Imagen 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E4FC3EB-5044-44DE-8A2E-3795AD849195}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16057072" y="10083535"/>
+          <a:ext cx="7772400" cy="3238499"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>191465</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>164250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>343865</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>164249</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Imagen 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3B55899-A4E6-4E25-936E-56184B0EA85F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16166251" y="13308750"/>
+          <a:ext cx="7772400" cy="3238499"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>259822</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>150963</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>412222</xdr:colOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>150962</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Imagen 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F002333D-C9C2-45C9-A718-D2D9FD9C6FCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16234608" y="16533963"/>
+          <a:ext cx="7772400" cy="3238499"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1451,10 +2347,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1468,10 +2364,10 @@
         <v>6</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1485,10 +2381,10 @@
         <v>25</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1502,10 +2398,10 @@
         <v>6</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1519,10 +2415,10 @@
         <v>6</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1536,10 +2432,10 @@
         <v>50</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1553,10 +2449,10 @@
         <v>50</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1570,10 +2466,10 @@
         <v>6</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1587,10 +2483,10 @@
         <v>6</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1604,10 +2500,10 @@
         <v>6</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1621,10 +2517,10 @@
         <v>6</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1638,10 +2534,10 @@
         <v>50</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1655,10 +2551,10 @@
         <v>6</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1672,15 +2568,15 @@
         <v>6</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>6</v>
@@ -1689,10 +2585,10 @@
         <v>6</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1706,10 +2602,10 @@
         <v>50</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:30" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -1739,7 +2635,7 @@
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
       <c r="U19" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="V19" s="9"/>
       <c r="W19" s="9"/>
@@ -1771,4 +2667,379 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{232E56B2-BA3E-44A2-B8C1-71FD82DA8185}">
+  <dimension ref="A1:AD19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="23">
+        <v>6</v>
+      </c>
+      <c r="C2" s="23">
+        <v>25</v>
+      </c>
+      <c r="D2" s="13">
+        <v>0.17430994</v>
+      </c>
+      <c r="E2" s="13">
+        <v>0.94</v>
+      </c>
+      <c r="F2" s="12">
+        <v>6.86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="23">
+        <v>5</v>
+      </c>
+      <c r="C3" s="23">
+        <v>25</v>
+      </c>
+      <c r="D3" s="13">
+        <v>0.21655086000000001</v>
+      </c>
+      <c r="E3" s="13">
+        <v>0.94</v>
+      </c>
+      <c r="F3" s="12">
+        <v>9.6300000000000008</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="23">
+        <v>4</v>
+      </c>
+      <c r="C4" s="23">
+        <v>250</v>
+      </c>
+      <c r="D4" s="13">
+        <v>0.15876303999999999</v>
+      </c>
+      <c r="E4" s="13">
+        <v>0.95333334000000003</v>
+      </c>
+      <c r="F4" s="12">
+        <v>10.54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="23">
+        <v>3</v>
+      </c>
+      <c r="C5" s="23">
+        <v>25</v>
+      </c>
+      <c r="D5" s="13">
+        <v>0.10254241</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0.96</v>
+      </c>
+      <c r="F5" s="12">
+        <v>10.87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="24">
+        <v>6</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="16">
+        <v>0.16795297000000001</v>
+      </c>
+      <c r="E6" s="16">
+        <v>0.94666667000000004</v>
+      </c>
+      <c r="F6" s="15">
+        <v>12.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="23">
+        <v>2</v>
+      </c>
+      <c r="C7" s="23">
+        <v>50</v>
+      </c>
+      <c r="D7" s="13">
+        <v>9.1158710000000004E-2</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0.95333334000000003</v>
+      </c>
+      <c r="F7" s="12">
+        <v>14.59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="24">
+        <v>5</v>
+      </c>
+      <c r="C8" s="24"/>
+      <c r="D8" s="16">
+        <v>0.21825589000000001</v>
+      </c>
+      <c r="E8" s="16">
+        <v>0.94</v>
+      </c>
+      <c r="F8" s="15">
+        <v>14.64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="24">
+        <v>4</v>
+      </c>
+      <c r="C9" s="24"/>
+      <c r="D9" s="16">
+        <v>0.14879745999999999</v>
+      </c>
+      <c r="E9" s="16">
+        <v>0.94666667000000004</v>
+      </c>
+      <c r="F9" s="15">
+        <v>15.35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="24">
+        <v>3</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="16">
+        <v>0.11040044</v>
+      </c>
+      <c r="E10" s="16">
+        <v>0.95333334000000003</v>
+      </c>
+      <c r="F10" s="15">
+        <v>17.239999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="24">
+        <v>2</v>
+      </c>
+      <c r="C11" s="24"/>
+      <c r="D11" s="16">
+        <v>0.10406952999999999</v>
+      </c>
+      <c r="E11" s="16">
+        <v>0.96</v>
+      </c>
+      <c r="F11" s="15">
+        <v>20.58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="25">
+        <v>5</v>
+      </c>
+      <c r="C12" s="25"/>
+      <c r="D12" s="19">
+        <v>0.61421276000000002</v>
+      </c>
+      <c r="E12" s="19">
+        <v>0.93333334000000001</v>
+      </c>
+      <c r="F12" s="18">
+        <v>29.26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="25">
+        <v>6</v>
+      </c>
+      <c r="C13" s="25"/>
+      <c r="D13" s="19">
+        <v>0.98352234999999999</v>
+      </c>
+      <c r="E13" s="19">
+        <v>0.91333333999999999</v>
+      </c>
+      <c r="F13" s="18">
+        <v>29.49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="25">
+        <v>3</v>
+      </c>
+      <c r="C14" s="25"/>
+      <c r="D14" s="19">
+        <v>0.21064245000000001</v>
+      </c>
+      <c r="E14" s="19">
+        <v>0.93333334000000001</v>
+      </c>
+      <c r="F14" s="18">
+        <v>29.65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="25">
+        <v>2</v>
+      </c>
+      <c r="C15" s="25"/>
+      <c r="D15" s="19">
+        <v>0.17135438</v>
+      </c>
+      <c r="E15" s="19">
+        <v>0.96</v>
+      </c>
+      <c r="F15" s="18">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="25">
+        <v>4</v>
+      </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="19">
+        <v>0.40213543000000002</v>
+      </c>
+      <c r="E16" s="19">
+        <v>0.94666667000000004</v>
+      </c>
+      <c r="F16" s="18">
+        <v>29.83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="21">
+        <v>0.10899017</v>
+      </c>
+      <c r="E17" s="21">
+        <v>0.94522229999999996</v>
+      </c>
+      <c r="F17" s="22">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="3"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="V19" s="9"/>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
+      <c r="Y19" s="9"/>
+      <c r="Z19" s="9"/>
+      <c r="AA19" s="9"/>
+      <c r="AB19" s="9"/>
+      <c r="AC19" s="9"/>
+      <c r="AD19" s="9"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F17">
+    <sortCondition ref="F1:F17"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización de los ultimos resultados
</commit_message>
<xml_diff>
--- a/ModeloFInal/resultados/RESUMEN EJECUCIÓN.xlsx
+++ b/ModeloFInal/resultados/RESUMEN EJECUCIÓN.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Desktop\Universidad\TFG\ModeloFinal\resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C691619-9FD0-44CA-8DF3-012E81B1CE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E7DFAF-6120-4E35-B5B2-247CCFA1F647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4048496F-68A2-4F9B-80AB-D81190A15522}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4048496F-68A2-4F9B-80AB-D81190A15522}"/>
   </bookViews>
   <sheets>
     <sheet name=" MAGIC Gamma Telescope" sheetId="1" r:id="rId1"/>
     <sheet name="IRIS" sheetId="2" r:id="rId2"/>
+    <sheet name="Neurona por grado" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="45">
   <si>
     <t>Polinomio</t>
   </si>
@@ -159,16 +160,26 @@
   </si>
   <si>
     <t>Tiempo_Promedio(s)</t>
+  </si>
+  <si>
+    <t>Legendre_Specialist</t>
+  </si>
+  <si>
+    <t>Chebyshev_Specialist</t>
+  </si>
+  <si>
+    <t>Shmaliy_Specialist</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000000"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
+    <numFmt numFmtId="169" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,6 +212,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="13">
@@ -320,7 +339,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
@@ -348,46 +367,107 @@
     <xf numFmtId="2" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -717,8 +797,8 @@
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>781050</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>73244</xdr:rowOff>
     </xdr:to>
@@ -767,8 +847,8 @@
       <xdr:rowOff>73800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>16650</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>778650</xdr:colOff>
       <xdr:row>53</xdr:row>
       <xdr:rowOff>127994</xdr:rowOff>
     </xdr:to>
@@ -817,8 +897,8 @@
       <xdr:rowOff>119025</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>23775</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>785775</xdr:colOff>
       <xdr:row>70</xdr:row>
       <xdr:rowOff>173219</xdr:rowOff>
     </xdr:to>
@@ -867,8 +947,8 @@
       <xdr:rowOff>11850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>40425</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>802425</xdr:colOff>
       <xdr:row>88</xdr:row>
       <xdr:rowOff>66044</xdr:rowOff>
     </xdr:to>
@@ -917,8 +997,8 @@
       <xdr:rowOff>57075</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>9450</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>771450</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>111269</xdr:rowOff>
     </xdr:to>
@@ -1017,8 +1097,8 @@
       <xdr:rowOff>73800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>150000</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>420711</xdr:colOff>
       <xdr:row>53</xdr:row>
       <xdr:rowOff>126131</xdr:rowOff>
     </xdr:to>
@@ -1167,8 +1247,8 @@
       <xdr:rowOff>180900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>114225</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>384936</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>42731</xdr:rowOff>
     </xdr:to>
@@ -1267,7 +1347,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
+      <xdr:colOff>647700</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>96583</xdr:rowOff>
     </xdr:to>
@@ -1316,8 +1396,8 @@
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>13259</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>689534</xdr:colOff>
       <xdr:row>55</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
@@ -1366,8 +1446,8 @@
       <xdr:rowOff>83325</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>63907</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>740182</xdr:colOff>
       <xdr:row>74</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
@@ -1417,7 +1497,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>92</xdr:row>
       <xdr:rowOff>145342</xdr:rowOff>
     </xdr:to>
@@ -1467,7 +1547,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>152399</xdr:colOff>
+      <xdr:colOff>66674</xdr:colOff>
       <xdr:row>111</xdr:row>
       <xdr:rowOff>68451</xdr:rowOff>
     </xdr:to>
@@ -2316,9 +2396,10 @@
     <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2335,8 +2416,26 @@
         <v>4</v>
       </c>
       <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q1" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="R1" s="28" t="s">
+        <v>2</v>
+      </c>
+      <c r="S1" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="T1" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="U1" s="28" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
@@ -2352,8 +2451,24 @@
       <c r="E2" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P2" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q2" s="29">
+        <v>3</v>
+      </c>
+      <c r="R2" s="29"/>
+      <c r="S2" s="30">
+        <v>0.30434684000000001</v>
+      </c>
+      <c r="T2" s="30">
+        <v>0.87939011</v>
+      </c>
+      <c r="U2" s="31">
+        <v>81.900000000000006</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
@@ -2369,8 +2484,24 @@
       <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P3" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q3" s="29">
+        <v>4</v>
+      </c>
+      <c r="R3" s="29"/>
+      <c r="S3" s="30">
+        <v>0.30622185000000002</v>
+      </c>
+      <c r="T3" s="30">
+        <v>0.87933753999999997</v>
+      </c>
+      <c r="U3" s="31">
+        <v>81.67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
@@ -2386,8 +2517,26 @@
       <c r="E4" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="32">
+        <v>5</v>
+      </c>
+      <c r="R4" s="32">
+        <v>50</v>
+      </c>
+      <c r="S4" s="33">
+        <v>0.30375583</v>
+      </c>
+      <c r="T4" s="33">
+        <v>0.87928494999999995</v>
+      </c>
+      <c r="U4" s="34">
+        <v>28.57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -2403,8 +2552,26 @@
       <c r="E5" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P5" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q5" s="32">
+        <v>4</v>
+      </c>
+      <c r="R5" s="32">
+        <v>50</v>
+      </c>
+      <c r="S5" s="33">
+        <v>0.29537918000000002</v>
+      </c>
+      <c r="T5" s="33">
+        <v>0.87828602</v>
+      </c>
+      <c r="U5" s="34">
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -2420,8 +2587,24 @@
       <c r="E6" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P6" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="35">
+        <v>2</v>
+      </c>
+      <c r="R6" s="35"/>
+      <c r="S6" s="36">
+        <v>0.30035550999999999</v>
+      </c>
+      <c r="T6" s="36">
+        <v>0.87828602</v>
+      </c>
+      <c r="U6" s="37">
+        <v>86.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -2437,8 +2620,26 @@
       <c r="E7" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q7" s="32">
+        <v>3</v>
+      </c>
+      <c r="R7" s="32">
+        <v>250</v>
+      </c>
+      <c r="S7" s="33">
+        <v>0.29774437999999998</v>
+      </c>
+      <c r="T7" s="33">
+        <v>0.87818085999999995</v>
+      </c>
+      <c r="U7" s="34">
+        <v>38.35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
@@ -2454,8 +2655,24 @@
       <c r="E8" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P8" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="29">
+        <v>2</v>
+      </c>
+      <c r="R8" s="29"/>
+      <c r="S8" s="30">
+        <v>0.30183972999999997</v>
+      </c>
+      <c r="T8" s="30">
+        <v>0.87697161000000001</v>
+      </c>
+      <c r="U8" s="31">
+        <v>85.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>5</v>
       </c>
@@ -2471,8 +2688,26 @@
       <c r="E9" s="7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P9" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q9" s="32">
+        <v>6</v>
+      </c>
+      <c r="R9" s="32">
+        <v>50</v>
+      </c>
+      <c r="S9" s="33">
+        <v>0.30920819999999999</v>
+      </c>
+      <c r="T9" s="33">
+        <v>0.87655099999999997</v>
+      </c>
+      <c r="U9" s="34">
+        <v>26.01</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>5</v>
       </c>
@@ -2488,8 +2723,24 @@
       <c r="E10" s="7" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P10" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="35">
+        <v>3</v>
+      </c>
+      <c r="R10" s="35"/>
+      <c r="S10" s="36">
+        <v>0.31767697</v>
+      </c>
+      <c r="T10" s="36">
+        <v>0.87549948</v>
+      </c>
+      <c r="U10" s="37">
+        <v>82.53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
@@ -2505,8 +2756,24 @@
       <c r="E11" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P11" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q11" s="29">
+        <v>5</v>
+      </c>
+      <c r="R11" s="29"/>
+      <c r="S11" s="30">
+        <v>0.32164161000000002</v>
+      </c>
+      <c r="T11" s="30">
+        <v>0.87518401999999995</v>
+      </c>
+      <c r="U11" s="31">
+        <v>82.92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>5</v>
       </c>
@@ -2522,8 +2789,24 @@
       <c r="E12" s="7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P12" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q12" s="35">
+        <v>4</v>
+      </c>
+      <c r="R12" s="35"/>
+      <c r="S12" s="36">
+        <v>0.33928202000000002</v>
+      </c>
+      <c r="T12" s="36">
+        <v>0.87465826000000002</v>
+      </c>
+      <c r="U12" s="37">
+        <v>83.93</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>8</v>
       </c>
@@ -2539,8 +2822,24 @@
       <c r="E13" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P13" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q13" s="29">
+        <v>6</v>
+      </c>
+      <c r="R13" s="29"/>
+      <c r="S13" s="30">
+        <v>0.39804403999999999</v>
+      </c>
+      <c r="T13" s="30">
+        <v>0.87439538000000006</v>
+      </c>
+      <c r="U13" s="31">
+        <v>84.23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>5</v>
       </c>
@@ -2556,8 +2855,26 @@
       <c r="E14" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P14" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q14" s="32">
+        <v>2</v>
+      </c>
+      <c r="R14" s="32">
+        <v>250</v>
+      </c>
+      <c r="S14" s="33">
+        <v>0.30798072999999998</v>
+      </c>
+      <c r="T14" s="33">
+        <v>0.87266036999999996</v>
+      </c>
+      <c r="U14" s="34">
+        <v>43.55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>7</v>
       </c>
@@ -2573,8 +2890,24 @@
       <c r="E15" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P15" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="35">
+        <v>5</v>
+      </c>
+      <c r="R15" s="35"/>
+      <c r="S15" s="36">
+        <v>0.41542330999999999</v>
+      </c>
+      <c r="T15" s="36">
+        <v>0.86798107999999996</v>
+      </c>
+      <c r="U15" s="37">
+        <v>85.39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
@@ -2589,6 +2922,22 @@
       </c>
       <c r="E16" s="6" t="s">
         <v>10</v>
+      </c>
+      <c r="P16" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q16" s="35">
+        <v>6</v>
+      </c>
+      <c r="R16" s="35"/>
+      <c r="S16" s="36">
+        <v>0.52014930999999998</v>
+      </c>
+      <c r="T16" s="36">
+        <v>0.85967404000000003</v>
+      </c>
+      <c r="U16" s="37">
+        <v>86.19</v>
       </c>
     </row>
     <row r="17" spans="1:30" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2660,8 +3009,8 @@
       <c r="J20" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E17">
-    <sortCondition descending="1" ref="E1:E17"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="P2:U16">
+    <sortCondition descending="1" ref="T2:T16"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2674,6 +3023,7 @@
   <dimension ref="A1:AD19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -2702,299 +3052,299 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="23">
-        <v>6</v>
-      </c>
-      <c r="C2" s="23">
-        <v>25</v>
-      </c>
-      <c r="D2" s="13">
-        <v>0.17430994</v>
-      </c>
-      <c r="E2" s="13">
-        <v>0.94</v>
-      </c>
-      <c r="F2" s="12">
-        <v>6.86</v>
+      <c r="A2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="21">
+        <v>2</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="23">
+        <v>0.16036922000000001</v>
+      </c>
+      <c r="E2" s="23">
+        <v>0.96666666999999995</v>
+      </c>
+      <c r="F2" s="16">
+        <v>27.81</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="23">
-        <v>5</v>
-      </c>
-      <c r="C3" s="23">
-        <v>25</v>
-      </c>
-      <c r="D3" s="13">
-        <v>0.21655086000000001</v>
-      </c>
-      <c r="E3" s="13">
-        <v>0.94</v>
-      </c>
-      <c r="F3" s="12">
-        <v>9.6300000000000008</v>
+      <c r="A3" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="20">
+        <v>2</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="26">
+        <v>0.14733107000000001</v>
+      </c>
+      <c r="E3" s="26">
+        <v>0.96</v>
+      </c>
+      <c r="F3" s="14">
+        <v>28.01</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="23">
+      <c r="B4" s="19">
+        <v>2</v>
+      </c>
+      <c r="C4" s="19">
+        <v>250</v>
+      </c>
+      <c r="D4" s="24">
+        <v>9.0500189999999994E-2</v>
+      </c>
+      <c r="E4" s="24">
+        <v>0.96</v>
+      </c>
+      <c r="F4" s="12">
+        <v>12.77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="25">
+        <v>0.13044389000000001</v>
+      </c>
+      <c r="E5" s="25">
+        <v>0.95666667000000005</v>
+      </c>
+      <c r="F5" s="18">
+        <v>29.62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="19">
+        <v>3</v>
+      </c>
+      <c r="C6" s="19">
+        <v>25</v>
+      </c>
+      <c r="D6" s="24">
+        <v>0.10173793</v>
+      </c>
+      <c r="E6" s="24">
+        <v>0.95333334000000003</v>
+      </c>
+      <c r="F6" s="12">
+        <v>10.77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="20">
         <v>4</v>
       </c>
-      <c r="C4" s="23">
-        <v>250</v>
-      </c>
-      <c r="D4" s="13">
-        <v>0.15876303999999999</v>
-      </c>
-      <c r="E4" s="13">
-        <v>0.95333334000000003</v>
-      </c>
-      <c r="F4" s="12">
-        <v>10.54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="C7" s="20"/>
+      <c r="D7" s="26">
+        <v>0.26089141999999999</v>
+      </c>
+      <c r="E7" s="26">
+        <v>0.94666667000000004</v>
+      </c>
+      <c r="F7" s="14">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="21">
+        <v>4</v>
+      </c>
+      <c r="C8" s="21"/>
+      <c r="D8" s="23">
+        <v>0.41056600999999998</v>
+      </c>
+      <c r="E8" s="23">
+        <v>0.94666667000000004</v>
+      </c>
+      <c r="F8" s="16">
+        <v>27.72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B9" s="19">
+        <v>4</v>
+      </c>
+      <c r="C9" s="19">
+        <v>25</v>
+      </c>
+      <c r="D9" s="24">
+        <v>0.14362887999999999</v>
+      </c>
+      <c r="E9" s="24">
+        <v>0.94666667000000004</v>
+      </c>
+      <c r="F9" s="12">
+        <v>9.02</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="20">
         <v>3</v>
       </c>
-      <c r="C5" s="23">
-        <v>25</v>
-      </c>
-      <c r="D5" s="13">
-        <v>0.10254241</v>
-      </c>
-      <c r="E5" s="13">
-        <v>0.96</v>
-      </c>
-      <c r="F5" s="12">
-        <v>10.87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="C10" s="20"/>
+      <c r="D10" s="26">
+        <v>0.18384238999999999</v>
+      </c>
+      <c r="E10" s="26">
+        <v>0.94</v>
+      </c>
+      <c r="F10" s="14">
+        <v>28.22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="21">
+        <v>5</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="23">
+        <v>0.44839108999999999</v>
+      </c>
+      <c r="E11" s="23">
+        <v>0.94</v>
+      </c>
+      <c r="F11" s="16">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="19">
+        <v>5</v>
+      </c>
+      <c r="C12" s="19">
+        <v>100</v>
+      </c>
+      <c r="D12" s="24">
+        <v>0.18543130999999999</v>
+      </c>
+      <c r="E12" s="24">
+        <v>0.94</v>
+      </c>
+      <c r="F12" s="12">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="19">
+        <v>6</v>
+      </c>
+      <c r="C13" s="19">
+        <v>50</v>
+      </c>
+      <c r="D13" s="24">
+        <v>0.18162381</v>
+      </c>
+      <c r="E13" s="24">
+        <v>0.94</v>
+      </c>
+      <c r="F13" s="12">
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="21">
+        <v>3</v>
+      </c>
+      <c r="C14" s="15"/>
+      <c r="D14" s="23">
+        <v>0.19892976000000001</v>
+      </c>
+      <c r="E14" s="23">
+        <v>0.93333334000000001</v>
+      </c>
+      <c r="F14" s="16">
+        <v>28.36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="24">
+      <c r="B15" s="20">
+        <v>5</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="26">
+        <v>0.33063315999999998</v>
+      </c>
+      <c r="E15" s="26">
+        <v>0.93333334000000001</v>
+      </c>
+      <c r="F15" s="14">
+        <v>28.15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="20">
         <v>6</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="16">
-        <v>0.16795297000000001</v>
-      </c>
-      <c r="E6" s="16">
-        <v>0.94666667000000004</v>
-      </c>
-      <c r="F6" s="15">
-        <v>12.05</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="23">
-        <v>2</v>
-      </c>
-      <c r="C7" s="23">
-        <v>50</v>
-      </c>
-      <c r="D7" s="13">
-        <v>9.1158710000000004E-2</v>
-      </c>
-      <c r="E7" s="13">
-        <v>0.95333334000000003</v>
-      </c>
-      <c r="F7" s="12">
-        <v>14.59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="24">
+      <c r="C16" s="13"/>
+      <c r="D16" s="26">
+        <v>0.46185271999999999</v>
+      </c>
+      <c r="E16" s="26">
+        <v>0.93333334000000001</v>
+      </c>
+      <c r="F16" s="14">
+        <v>28.08</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="16">
-        <v>0.21825589000000001</v>
-      </c>
-      <c r="E8" s="16">
-        <v>0.94</v>
-      </c>
-      <c r="F8" s="15">
-        <v>14.64</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="24">
-        <v>4</v>
-      </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="16">
-        <v>0.14879745999999999</v>
-      </c>
-      <c r="E9" s="16">
-        <v>0.94666667000000004</v>
-      </c>
-      <c r="F9" s="15">
-        <v>15.35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="24">
-        <v>3</v>
-      </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="16">
-        <v>0.11040044</v>
-      </c>
-      <c r="E10" s="16">
-        <v>0.95333334000000003</v>
-      </c>
-      <c r="F10" s="15">
-        <v>17.239999999999998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="24">
-        <v>2</v>
-      </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="16">
-        <v>0.10406952999999999</v>
-      </c>
-      <c r="E11" s="16">
-        <v>0.96</v>
-      </c>
-      <c r="F11" s="15">
-        <v>20.58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="25">
-        <v>5</v>
-      </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="19">
-        <v>0.61421276000000002</v>
-      </c>
-      <c r="E12" s="19">
-        <v>0.93333334000000001</v>
-      </c>
-      <c r="F12" s="18">
-        <v>29.26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="25">
+      <c r="B17" s="21">
         <v>6</v>
       </c>
-      <c r="C13" s="25"/>
-      <c r="D13" s="19">
-        <v>0.98352234999999999</v>
-      </c>
-      <c r="E13" s="19">
-        <v>0.91333333999999999</v>
-      </c>
-      <c r="F13" s="18">
-        <v>29.49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="25">
-        <v>3</v>
-      </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="19">
-        <v>0.21064245000000001</v>
-      </c>
-      <c r="E14" s="19">
-        <v>0.93333334000000001</v>
-      </c>
-      <c r="F14" s="18">
-        <v>29.65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="25">
-        <v>2</v>
-      </c>
-      <c r="C15" s="25"/>
-      <c r="D15" s="19">
-        <v>0.17135438</v>
-      </c>
-      <c r="E15" s="19">
-        <v>0.96</v>
-      </c>
-      <c r="F15" s="18">
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="25">
-        <v>4</v>
-      </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="19">
-        <v>0.40213543000000002</v>
-      </c>
-      <c r="E16" s="19">
-        <v>0.94666667000000004</v>
-      </c>
-      <c r="F16" s="18">
-        <v>29.83</v>
-      </c>
-    </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A17" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="21">
-        <v>0.10899017</v>
-      </c>
-      <c r="E17" s="21">
-        <v>0.94522229999999996</v>
-      </c>
-      <c r="F17" s="22">
-        <v>34.5</v>
+      <c r="C17" s="15"/>
+      <c r="D17" s="23">
+        <v>0.51323213000000001</v>
+      </c>
+      <c r="E17" s="23">
+        <v>0.92</v>
+      </c>
+      <c r="F17" s="16">
+        <v>28.03</v>
       </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.25">
@@ -3037,9 +3387,216 @@
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F17">
-    <sortCondition ref="F1:F17"/>
+    <sortCondition descending="1" ref="E1:E17"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4572D35A-6012-47F1-816E-5469A843D6C0}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="38" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="39">
+        <v>3</v>
+      </c>
+      <c r="C2" s="39"/>
+      <c r="D2" s="40">
+        <v>8.7195999999999996E-2</v>
+      </c>
+      <c r="E2" s="40">
+        <v>0.95</v>
+      </c>
+      <c r="F2" s="41">
+        <v>22.66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="42">
+        <v>3</v>
+      </c>
+      <c r="C3" s="42"/>
+      <c r="D3" s="43">
+        <v>0.13528200000000001</v>
+      </c>
+      <c r="E3" s="43">
+        <v>0.95</v>
+      </c>
+      <c r="F3" s="44">
+        <v>22.55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="42">
+        <v>5</v>
+      </c>
+      <c r="C4" s="42"/>
+      <c r="D4" s="43">
+        <v>0.117781</v>
+      </c>
+      <c r="E4" s="43">
+        <v>0.95333299999999999</v>
+      </c>
+      <c r="F4" s="44">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="39">
+        <v>5</v>
+      </c>
+      <c r="C5" s="39"/>
+      <c r="D5" s="40">
+        <v>0.143375</v>
+      </c>
+      <c r="E5" s="40">
+        <v>0.94666700000000004</v>
+      </c>
+      <c r="F5" s="41">
+        <v>22.61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="39">
+        <v>10</v>
+      </c>
+      <c r="C6" s="39"/>
+      <c r="D6" s="40">
+        <v>0.30736999999999998</v>
+      </c>
+      <c r="E6" s="40">
+        <v>0.94666700000000004</v>
+      </c>
+      <c r="F6" s="41">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="42">
+        <v>10</v>
+      </c>
+      <c r="C7" s="42"/>
+      <c r="D7" s="43">
+        <v>0.92090899999999998</v>
+      </c>
+      <c r="E7" s="43">
+        <v>0.94</v>
+      </c>
+      <c r="F7" s="44">
+        <v>22.02</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="45">
+        <v>3</v>
+      </c>
+      <c r="C8" s="45">
+        <v>50</v>
+      </c>
+      <c r="D8" s="46">
+        <v>0.40217000000000003</v>
+      </c>
+      <c r="E8" s="46">
+        <v>0.8</v>
+      </c>
+      <c r="F8" s="47">
+        <v>20.22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="45">
+        <v>5</v>
+      </c>
+      <c r="C9" s="45">
+        <v>25</v>
+      </c>
+      <c r="D9" s="46">
+        <v>0.53414300000000003</v>
+      </c>
+      <c r="E9" s="46">
+        <v>0.73333300000000001</v>
+      </c>
+      <c r="F9" s="47">
+        <v>20.64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="45">
+        <v>10</v>
+      </c>
+      <c r="C10" s="45">
+        <v>250</v>
+      </c>
+      <c r="D10" s="46">
+        <v>3.0194429999999999</v>
+      </c>
+      <c r="E10" s="46">
+        <v>0.68</v>
+      </c>
+      <c r="F10" s="47">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G13" s="27"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>